<commit_message>
📊 Horarios actualizados Línea 141 - 2551
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,166 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:42:02</t>
+          <t>Última actualización: 03:20:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>03:20:25</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>03:48</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>03:20:25</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>04:01</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>41</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>03:20:25</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:46</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>86</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03:20:25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:53</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>93</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>03:20:25</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>05:16</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>116</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -454,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,14 +619,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:42:02</t>
+          <t>Última actualización: 03:20:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>03:20:25</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>04:46</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>86</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -502,7 +706,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:42:02</t>
+          <t>Última actualización: 03:20:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2552
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:20:25</t>
+          <t>Última actualización: 04:51:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:20:25</t>
+          <t>04:51:13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:20:25</t>
+          <t>04:51:13</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:01</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:20:25</t>
+          <t>04:51:13</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:46</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>86</v>
+        <v>31</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:20:25</t>
+          <t>04:51:13</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>93</v>
+        <v>53</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,23 +573,223 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:20:25</t>
+          <t>04:51:13</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:16</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>116</v>
+        <v>56</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>04:51:13</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>70</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>04:51:13</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06:09</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>78</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:51:13</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>81</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:51:13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>99</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:51:13</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:36</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>105</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:51:13</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>108</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:51:13</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>110</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04:51:13</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>110</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -619,7 +819,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:20:25</t>
+          <t>Última actualización: 04:51:13</t>
         </is>
       </c>
     </row>
@@ -660,12 +860,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:20:25</t>
+          <t>04:51:13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:46</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -674,7 +874,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -706,7 +906,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:20:25</t>
+          <t>Última actualización: 04:51:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2553
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:51:13</t>
+          <t>Última actualización: 05:41:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>105</v>
+        <v>78</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>108</v>
+        <v>81</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,23 +773,98 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>05:41:12</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07:27</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>106</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>05:41:12</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>111</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>05:41:12</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>116</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -806,7 +881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -819,14 +894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:51:13</t>
+          <t>Última actualización: 05:41:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -860,7 +935,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:51:13</t>
+          <t>05:41:12</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -874,9 +949,59 @@
         </is>
       </c>
       <c r="D6" t="n">
+        <v>31</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:41:12</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
         <v>81</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05:41:12</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>111</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -906,7 +1031,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:51:13</t>
+          <t>Última actualización: 05:41:12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2554
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:41:12</t>
+          <t>Última actualización: 06:32:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>105</v>
+        <v>79</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,12 +798,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,23 +848,48 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>06:32:42</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>113</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -894,7 +919,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:41:12</t>
+          <t>Última actualización: 06:32:42</t>
         </is>
       </c>
     </row>
@@ -935,12 +960,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -949,7 +974,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -960,21 +985,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>81</v>
+        <v>59</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -985,21 +1010,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:41:12</t>
+          <t>06:32:42</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>111</v>
+        <v>79</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1018,7 +1043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1031,14 +1056,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:41:12</t>
+          <t>Última actualización: 06:32:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:32:42</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>76</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2555
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:32:42</t>
+          <t>Última actualización: 07:21:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>06:32:42</t>
+          <t>07:21:33</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>06:32:42</t>
+          <t>07:21:33</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:32:42</t>
+          <t>07:21:33</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>59</v>
+        <v>6</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:32:42</t>
+          <t>07:21:33</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>64</v>
+        <v>10</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:32:42</t>
+          <t>07:21:33</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>72</v>
+        <v>15</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:32:42</t>
+          <t>07:21:33</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>79</v>
+        <v>23</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:32:42</t>
+          <t>07:21:33</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>07:45</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>94</v>
+        <v>24</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:32:42</t>
+          <t>07:21:33</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>30</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:32:42</t>
+          <t>07:21:33</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>109</v>
+        <v>40</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,23 +873,223 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08:06</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>45</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>58</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>06:32:42</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>109</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>08:25</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>113</v>
-      </c>
-      <c r="E22" t="inlineStr">
+      <c r="D25" t="n">
+        <v>64</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>83</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>84</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>103</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>105</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>115</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -906,7 +1106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -919,14 +1119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:32:42</t>
+          <t>Última actualización: 07:21:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -985,7 +1185,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:32:42</t>
+          <t>07:21:33</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -999,7 +1199,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>59</v>
+        <v>10</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1010,7 +1210,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:32:42</t>
+          <t>07:21:33</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1024,9 +1224,84 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>79</v>
+        <v>30</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>83</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>84</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>105</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1043,7 +1318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1056,14 +1331,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:32:42</t>
+          <t>Última actualización: 07:21:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -1116,6 +1391,81 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>28</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>77</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:21:33</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>101</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2556
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:21:33</t>
+          <t>Última actualización: 08:03:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:21:33</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07:21:33</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -948,21 +948,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>07:21:33</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>08:25</t>
+          <t>08:23</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,21 +973,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07:21:33</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:25</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:21:33</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:21:33</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>07:21:33</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>105</v>
+        <v>42</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,23 +1073,298 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>07:21:33</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>61</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>61</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>63</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>09:16</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>115</v>
-      </c>
-      <c r="E30" t="inlineStr">
+      <c r="D33" t="n">
+        <v>73</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>73</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>78</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>81</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>91</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>92</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>101</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>112</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>117</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1106,7 +1381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1119,14 +1394,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:21:33</t>
+          <t>Última actualización: 08:03:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1510,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:21:33</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1249,7 +1524,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>83</v>
+        <v>41</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1260,7 +1535,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:21:33</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1274,7 +1549,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1285,7 +1560,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:21:33</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1299,9 +1574,34 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>112</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1318,7 +1618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1331,14 +1631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:21:33</t>
+          <t>Última actualización: 08:03:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1722,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07:21:33</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1436,7 +1736,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1466,6 +1766,56 @@
       <c r="E9" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>60</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>85</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2557
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:03:30</t>
+          <t>Última actualización: 08:46:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:46</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>78</v>
+        <v>30</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:21</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>91</v>
+        <v>35</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>92</v>
+        <v>38</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>101</v>
+        <v>48</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>112</v>
+        <v>49</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,23 +1348,273 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>58</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>65</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>68</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>08:03:30</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>112</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>08:03:30</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D41" t="n">
+      <c r="D45" t="n">
         <v>117</v>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>78</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>79</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>89</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>98</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>108</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>118</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1381,7 +1631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1394,14 +1644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:03:30</t>
+          <t>Última actualización: 08:46:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1560,21 +1810,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:46</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1585,23 +1835,73 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>68</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>08:03:30</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>09:55</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D14" t="n">
         <v>112</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1618,7 +1918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1631,14 +1931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:03:30</t>
+          <t>Última actualización: 08:46:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1747,7 +2047,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:21:33</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1761,7 +2061,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>101</v>
+        <v>16</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1797,23 +2097,123 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>41</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>08:03:30</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>09:28</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>85</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>10:17</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>91</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>103</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>116</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2558
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:46:39</t>
+          <t>Última actualización: 09:04:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 46</t>
+          <t>Total filas: 55</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1203,16 +1203,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1278,16 +1278,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>48</v>
+        <v>13</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:21</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>68</v>
+        <v>31</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>112</v>
+        <v>58</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>117</v>
+        <v>41</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1478,16 +1478,16 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1503,16 +1503,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>10:05</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>89</v>
+        <v>51</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:02</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>108</v>
+        <v>58</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,23 +1598,248 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>09:04:03</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>60</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>08:46:39</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>79</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>09:04:03</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>71</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>98</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>09:04:03</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>81</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>09:04:03</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>90</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>09:04:03</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
         <is>
           <t>10:44</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D51" t="n">
-        <v>118</v>
-      </c>
-      <c r="E51" t="inlineStr">
+      <c r="D57" t="n">
+        <v>100</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>09:04:03</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>111</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>09:04:03</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>113</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>09:04:03</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>11:01</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>117</v>
+      </c>
+      <c r="E60" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1631,7 +1856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1644,14 +1869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:46:39</t>
+          <t>Última actualización: 09:04:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1860,21 +2085,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1885,23 +2110,48 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>68</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>09:04:03</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>09:55</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>112</v>
-      </c>
-      <c r="E14" t="inlineStr">
+      <c r="D15" t="n">
+        <v>51</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1918,7 +2168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1931,14 +2181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:46:39</t>
+          <t>Última actualización: 09:04:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2097,37 +2347,37 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>09:27</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>09:28</t>
+          <t>09:27</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2136,7 +2386,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>85</v>
+        <v>41</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2147,25 +2397,25 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10:17</t>
+          <t>09:28</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>91</v>
+        <v>24</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
@@ -2177,43 +2427,143 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10:29</t>
+          <t>10:17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>09:04:03</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>74</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>08:46:39</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>103</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>09:04:03</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>86</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:46:39</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>10:42</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D18" t="n">
         <v>116</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>09:04:03</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>99</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2559
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:04:03</t>
+          <t>Última actualización: 10:21:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 55</t>
+          <t>Total filas: 70</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>98</v>
+        <v>3</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>90</v>
+        <v>5</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:34</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>100</v>
+        <v>13</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>111</v>
+        <v>22</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1803,16 +1803,16 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>10:57</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,23 +1823,398 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>30</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>34</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>35</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>09:04:03</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>113</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
         <is>
           <t>11:01</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D60" t="n">
-        <v>117</v>
-      </c>
-      <c r="E60" t="inlineStr">
+      <c r="D64" t="n">
+        <v>40</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>43</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>11:07</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>46</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>11:09</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>48</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>62</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>73</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>83</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>84</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>93</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>94</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>12:03</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>102</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>114</v>
+      </c>
+      <c r="E75" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1856,7 +2231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1869,14 +2244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:04:03</t>
+          <t>Última actualización: 10:21:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2152,6 +2527,56 @@
         <v>51</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>73</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>83</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2168,7 +2593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2181,14 +2606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:04:03</t>
+          <t>Última actualización: 10:21:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2897,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2486,7 +2911,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>103</v>
+        <v>8</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2522,7 +2947,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2536,7 +2961,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>116</v>
+        <v>21</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2566,6 +2991,31 @@
       <c r="E19" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:22</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>61</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2560
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:21:55</t>
+          <t>Última actualización: 11:07:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 70</t>
+          <t>Total filas: 86</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>11:09</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2028,16 +2028,16 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>11:23</t>
+          <t>11:09</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>73</v>
+        <v>8</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2078,16 +2078,16 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:23</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>11:24</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>84</v>
+        <v>17</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2128,16 +2128,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:34</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>94</v>
+        <v>28</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>102</v>
+        <v>29</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,23 +2198,423 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>34</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
           <t>10:21:55</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>83</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>84</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>38</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>47</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>48</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>10:21:55</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>12:03</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>102</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>57</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D75" t="n">
-        <v>114</v>
-      </c>
-      <c r="E75" t="inlineStr">
+      <c r="D83" t="n">
+        <v>68</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>78</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>85</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>87</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>12:41</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>94</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>97</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>99</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>108</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>118</v>
+      </c>
+      <c r="E91" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2231,7 +2631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2244,14 +2644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:21:55</t>
+          <t>Última actualización: 11:07:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2560,23 +2960,98 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>28</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>10:21:55</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>11:44</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D18" t="n">
         <v>83</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>38</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>108</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2593,7 +3068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2606,14 +3081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:21:55</t>
+          <t>Última actualización: 11:07:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3014,6 +3489,31 @@
         <v>61</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>16</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2561
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E91"/>
+  <dimension ref="A1:E102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:07:14</t>
+          <t>Última actualización: 11:54:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 86</t>
+          <t>Total filas: 97</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,7 +2298,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>11:54:49</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2312,7 +2312,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>11:54:49</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>11:54:49</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>11:54:49</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>11:54:49</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>78</v>
+        <v>21</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>11:54:49</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>85</v>
+        <v>30</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2478,16 +2478,16 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>11:54:49</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>12:41</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>94</v>
+        <v>37</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2528,16 +2528,16 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>11:54:49</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>99</v>
+        <v>40</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>11:54:49</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>108</v>
+        <v>42</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2603,18 +2603,293 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
+          <t>12:41</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>94</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>50</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>52</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>60</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>108</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>70</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>11:07:13</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
           <t>13:05</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C97" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D91" t="n">
+      <c r="D97" t="n">
         <v>118</v>
       </c>
-      <c r="E91" t="inlineStr">
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>81</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>90</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>91</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>97</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>110</v>
+      </c>
+      <c r="E102" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2631,7 +2906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2644,14 +2919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:07:14</t>
+          <t>Última actualización: 11:54:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3035,23 +3310,73 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>60</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>11:07:13</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>12:55</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="D21" t="n">
         <v>108</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>97</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3068,7 +3393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3081,14 +3406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:07:14</t>
+          <t>Última actualización: 11:54:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3516,6 +3841,56 @@
       <c r="E21" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>88</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>115</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2562
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E102"/>
+  <dimension ref="A1:E114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:54:49</t>
+          <t>Última actualización: 12:28:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 97</t>
+          <t>Total filas: 109</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>85</v>
+        <v>4</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,7 +2548,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2562,7 +2562,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2598,12 +2598,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>12:41</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2612,7 +2612,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>94</v>
+        <v>9</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:41</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>50</v>
+        <v>94</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:46</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,12 +2698,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>11:54:49</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>108</v>
+        <v>60</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,12 +2748,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>11:54:49</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2762,7 +2762,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>118</v>
+        <v>70</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>81</v>
+        <v>37</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:08</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>91</v>
+        <v>47</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>97</v>
+        <v>56</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2878,18 +2878,318 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>91</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>13:29</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>61</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>97</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>64</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>11:54:49</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
           <t>13:44</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C106" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D102" t="n">
+      <c r="D106" t="n">
         <v>110</v>
       </c>
-      <c r="E102" t="inlineStr">
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>77</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>87</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>88</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>96</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>106</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>106</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>109</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>117</v>
+      </c>
+      <c r="E114" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2906,7 +3206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2919,14 +3219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:54:49</t>
+          <t>Última actualización: 12:28:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3635,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3349,7 +3649,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3377,6 +3677,31 @@
         <v>97</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>64</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3393,7 +3718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3406,14 +3731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:54:49</t>
+          <t>Última actualización: 12:28:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -3872,23 +4197,73 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>55</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>11:54:49</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>13:49</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D24" t="n">
         <v>115</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>82</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2563
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E114"/>
+  <dimension ref="A1:E122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:28:03</t>
+          <t>Última actualización: 12:59:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 109</t>
+          <t>Total filas: 117</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2748,12 +2748,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2762,7 +2762,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,12 +2773,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>12:28:03</t>
+          <t>11:54:49</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2787,7 +2787,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>37</v>
+        <v>70</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2803,16 +2803,16 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>13:08</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2828,16 +2828,16 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:08</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>12:28:03</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>56</v>
+        <v>16</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,12 +2898,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>12:28:03</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>13:29</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2912,7 +2912,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:29</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>97</v>
+        <v>61</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,12 +2948,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>12:28:03</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2962,7 +2962,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>110</v>
+        <v>64</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,12 +2998,12 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>12:28:03</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>77</v>
+        <v>45</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3028,16 +3028,16 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>12:28:03</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>88</v>
+        <v>56</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>12:28:03</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>13:56</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>96</v>
+        <v>57</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>12:28:03</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>106</v>
+        <v>65</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>12:28:03</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>12:28:03</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,23 +3173,223 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
+          <t>12:59:47</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>75</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>12:59:47</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>77</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
           <t>12:28:03</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>109</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>12:59:47</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>85</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>12:28:03</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
         <is>
           <t>14:25</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C118" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D114" t="n">
+      <c r="D118" t="n">
         <v>117</v>
       </c>
-      <c r="E114" t="inlineStr">
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>12:59:47</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>92</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>12:59:47</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>95</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>12:59:47</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>105</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>12:59:47</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>115</v>
+      </c>
+      <c r="E122" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3206,7 +3406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3219,14 +3419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:28:03</t>
+          <t>Última actualización: 12:59:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -3660,7 +3860,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3674,7 +3874,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3702,6 +3902,56 @@
         <v>64</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>12:59:47</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>95</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>12:59:47</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>115</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3718,7 +3968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3731,14 +3981,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:28:03</t>
+          <t>Última actualización: 12:59:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4422,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4186,7 +4436,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>88</v>
+        <v>23</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4222,7 +4472,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:54:49</t>
+          <t>12:59:47</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4236,7 +4486,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4266,6 +4516,31 @@
       <c r="E25" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>12:59:47</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>103</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2564
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E122"/>
+  <dimension ref="A1:E128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:59:47</t>
+          <t>Última actualización: 13:41:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 117</t>
+          <t>Total filas: 123</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:41</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,12 +3023,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>12:28:03</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>77</v>
+        <v>3</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>13:56</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>65</v>
+        <v>15</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>72</v>
+        <v>23</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3187,7 +3187,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,12 +3223,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>12:28:03</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>109</v>
+        <v>35</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,12 +3273,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>12:28:03</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>117</v>
+        <v>43</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>12:28:03</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>92</v>
+        <v>117</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>95</v>
+        <v>50</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>105</v>
+        <v>53</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,23 +3373,173 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>63</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>13:41:42</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
           <t>14:54</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
+      <c r="C123" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D122" t="n">
-        <v>115</v>
-      </c>
-      <c r="E122" t="inlineStr">
+      <c r="D123" t="n">
+        <v>73</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>13:41:42</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>83</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>13:41:42</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>86</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>13:41:42</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>94</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>13:41:42</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>103</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>13:41:42</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>113</v>
+      </c>
+      <c r="E128" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3406,7 +3556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3419,14 +3569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:59:47</t>
+          <t>Última actualización: 13:41:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -3910,7 +4060,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3924,7 +4074,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>95</v>
+        <v>53</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -3935,7 +4085,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3949,9 +4099,59 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>13:41:42</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>83</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>13:41:42</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>113</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3968,7 +4168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3981,14 +4181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:59:47</t>
+          <t>Última actualización: 13:41:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4672,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4486,7 +4686,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4522,7 +4722,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:59:47</t>
+          <t>13:41:42</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4536,11 +4736,36 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>13:41:42</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>101</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2565
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E128"/>
+  <dimension ref="A1:E136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:41:42</t>
+          <t>Última actualización: 14:21:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 123</t>
+          <t>Total filas: 131</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>43</v>
+        <v>3</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3362,7 +3362,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>53</v>
+        <v>13</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3387,7 +3387,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>63</v>
+        <v>23</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3412,7 +3412,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>86</v>
+        <v>43</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>94</v>
+        <v>45</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3503,16 +3503,16 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,23 +3523,223 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>54</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>14:21:40</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>63</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>14:21:40</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
           <t>15:34</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr">
+      <c r="C130" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D128" t="n">
+      <c r="D130" t="n">
+        <v>73</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>14:21:40</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>83</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>14:21:40</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>15:49</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>88</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>14:21:40</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>94</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>14:21:40</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>95</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>14:21:40</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>103</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>14:21:40</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
         <v>113</v>
       </c>
-      <c r="E128" t="inlineStr">
+      <c r="E136" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3569,7 +3769,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:41:42</t>
+          <t>Última actualización: 14:21:40</t>
         </is>
       </c>
     </row>
@@ -4060,7 +4260,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4074,7 +4274,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>53</v>
+        <v>13</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4085,7 +4285,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4099,7 +4299,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4110,7 +4310,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4124,7 +4324,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4135,7 +4335,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4149,7 +4349,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>113</v>
+        <v>73</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4168,7 +4368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4181,14 +4381,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:41:42</t>
+          <t>Última actualización: 14:21:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -4722,7 +4922,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4736,7 +4936,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4747,7 +4947,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:41:42</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4761,11 +4961,36 @@
         </is>
       </c>
       <c r="D27" t="n">
+        <v>61</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>14:21:40</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
         <v>101</v>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>L6173</t>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2566
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E136"/>
+  <dimension ref="A1:E145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:21:40</t>
+          <t>Última actualización: 14:57:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 131</t>
+          <t>Total filas: 140</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>14:21:40</t>
+          <t>14:57:19</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>14:21:40</t>
+          <t>14:57:19</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3462,7 +3462,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>43</v>
+        <v>7</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>14:21:40</t>
+          <t>14:57:19</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3487,7 +3487,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>14:21:40</t>
+          <t>14:57:19</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>14:21:40</t>
+          <t>14:57:19</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3562,7 +3562,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>14:21:40</t>
+          <t>14:57:19</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>83</v>
+        <v>38</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>14:21:40</t>
+          <t>14:57:19</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>15:49</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>14:21:40</t>
+          <t>14:57:19</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>94</v>
+        <v>47</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3678,16 +3678,16 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:49</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>14:21:40</t>
+          <t>14:57:19</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>103</v>
+        <v>54</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,23 +3723,248 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
+          <t>14:57:19</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>58</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
           <t>14:21:40</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr">
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>95</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>14:57:19</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>60</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>14:57:19</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>67</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>14:57:19</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
         <is>
           <t>16:14</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr">
+      <c r="C140" t="inlineStr">
         <is>
           <t>17X38_ROMERO</t>
         </is>
       </c>
-      <c r="D136" t="n">
-        <v>113</v>
-      </c>
-      <c r="E136" t="inlineStr">
+      <c r="D140" t="n">
+        <v>77</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>14:57:19</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>87</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>14:57:19</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>97</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>14:57:19</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>98</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>14:57:19</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>107</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>14:57:19</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>118</v>
+      </c>
+      <c r="E145" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3756,7 +3981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3769,14 +3994,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:21:40</t>
+          <t>Última actualización: 14:57:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -4310,7 +4535,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>14:21:40</t>
+          <t>14:57:19</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4324,7 +4549,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>43</v>
+        <v>7</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4352,6 +4577,31 @@
         <v>73</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>14:57:19</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>38</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4368,7 +4618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4381,14 +4631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:21:40</t>
+          <t>Última actualización: 14:57:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -4972,25 +5222,100 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>14:57:19</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>26</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>14:21:40</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>16:02</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D29" t="n">
         <v>101</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>14:57:19</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>66</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>14:57:19</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>93</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2567
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E145"/>
+  <dimension ref="A1:E153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:57:19</t>
+          <t>Última actualización: 15:39:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 140</t>
+          <t>Total filas: 148</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>14:57:19</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>44</v>
+        <v>1</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>14:57:19</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>14:21:40</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>15:49</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>88</v>
+        <v>5</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,12 +3698,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>14:57:19</t>
+          <t>14:21:40</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:49</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -3712,7 +3712,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>14:57:19</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>14:21:40</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>95</v>
+        <v>16</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,12 +3773,12 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>14:57:19</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3803,16 +3803,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>14:57:19</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>14:57:19</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>87</v>
+        <v>35</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:57:19</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:16</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:57:19</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>98</v>
+        <v>45</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>14:57:19</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>107</v>
+        <v>55</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,23 +3948,223 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>14:57:19</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>56</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>15:39:36</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>65</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>15:39:36</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
           <t>16:55</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr">
+      <c r="C147" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D145" t="n">
-        <v>118</v>
-      </c>
-      <c r="E145" t="inlineStr">
+      <c r="D147" t="n">
+        <v>76</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>15:39:36</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>85</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>15:39:36</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>95</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>15:39:36</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>105</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>15:39:36</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>112</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>15:39:36</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>116</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>15:39:36</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>117</v>
+      </c>
+      <c r="E153" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3981,7 +4181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3994,14 +4194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:57:19</t>
+          <t>Última actualización: 15:39:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -4602,6 +4802,56 @@
         <v>38</v>
       </c>
       <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>15:39:36</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>15:39:36</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>95</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4618,7 +4868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4631,14 +4881,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:57:19</t>
+          <t>Última actualización: 15:39:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -5247,7 +5497,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>14:21:40</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5261,7 +5511,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>101</v>
+        <v>23</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5297,7 +5547,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:57:19</t>
+          <t>15:39:36</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5311,11 +5561,36 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>15:39:36</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>103</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2568
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E153"/>
+  <dimension ref="A1:E165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:39:36</t>
+          <t>Última actualización: 16:28:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 148</t>
+          <t>Total filas: 160</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3962,7 +3962,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:43</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>65</v>
+        <v>15</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>85</v>
+        <v>23</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>95</v>
+        <v>27</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4078,16 +4078,16 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>112</v>
+        <v>37</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4128,16 +4128,16 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>116</v>
+        <v>95</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,23 +4148,323 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>47</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>56</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>17:26</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>58</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>62</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
           <t>15:39:36</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr">
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>112</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>67</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>67</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>15:39:36</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
         <is>
           <t>17:36</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr">
+      <c r="C160" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D153" t="n">
+      <c r="D160" t="n">
         <v>117</v>
       </c>
-      <c r="E153" t="inlineStr">
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>77</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>87</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>17:58</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>90</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>107</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>117</v>
+      </c>
+      <c r="E165" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4181,7 +4481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4194,14 +4494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:39:36</t>
+          <t>Última actualización: 16:28:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -4852,6 +5152,106 @@
         <v>95</v>
       </c>
       <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>47</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>77</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>87</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>107</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4868,7 +5268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4881,14 +5281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:39:36</t>
+          <t>Última actualización: 16:28:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -5547,7 +5947,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5561,7 +5961,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -5589,6 +5989,31 @@
         <v>103</v>
       </c>
       <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>55</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2569
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E165"/>
+  <dimension ref="A1:E177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:28:16</t>
+          <t>Última actualización: 16:58:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 160</t>
+          <t>Total filas: 172</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4087,7 +4087,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>85</v>
+        <v>6</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>95</v>
+        <v>16</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4173,12 +4173,12 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:23</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4203,16 +4203,16 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>17:26</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,12 +4248,12 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>112</v>
+        <v>62</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>67</v>
+        <v>33</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:34</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>117</v>
+        <v>67</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4353,16 +4353,16 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>87</v>
+        <v>38</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>17:58</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>90</v>
+        <v>46</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4428,16 +4428,16 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>107</v>
+        <v>77</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,23 +4448,323 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>56</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
           <t>16:28:16</t>
         </is>
       </c>
-      <c r="B165" t="inlineStr">
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>87</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>17:58</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>90</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>18:03</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>65</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>76</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>107</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>86</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
         <is>
           <t>18:25</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr">
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>87</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D165" t="n">
+      <c r="D173" t="n">
         <v>117</v>
       </c>
-      <c r="E165" t="inlineStr">
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>96</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>98</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>18:43</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>105</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>116</v>
+      </c>
+      <c r="E177" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4481,7 +4781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4494,14 +4794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:28:16</t>
+          <t>Última actualización: 16:58:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -5135,7 +5435,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5149,7 +5449,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>95</v>
+        <v>16</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5185,12 +5485,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -5199,7 +5499,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>77</v>
+        <v>46</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5215,16 +5515,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5235,23 +5535,98 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>56</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>16:28:16</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>87</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>76</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16:28:16</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
         <is>
           <t>18:15</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="D37" t="n">
         <v>107</v>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5268,7 +5643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5281,14 +5656,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:28:16</t>
+          <t>Última actualización: 16:58:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5972,7 +6347,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>15:39:36</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5986,7 +6361,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>103</v>
+        <v>24</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -6014,6 +6389,31 @@
         <v>55</v>
       </c>
       <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>106</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2570
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E177"/>
+  <dimension ref="A1:E187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:58:56</t>
+          <t>Última actualización: 17:35:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 172</t>
+          <t>Total filas: 182</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4362,7 +4362,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>46</v>
+        <v>9</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4448,7 +4448,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -4462,7 +4462,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>18:14</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>76</v>
+        <v>29</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,12 +4573,12 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>107</v>
+        <v>39</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>87</v>
+        <v>49</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4658,11 +4658,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:32</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>98</v>
+        <v>57</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>18:43</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>105</v>
+        <v>59</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,23 +4748,273 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
+          <t>17:35:45</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>61</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
           <t>16:58:56</t>
         </is>
       </c>
-      <c r="B177" t="inlineStr">
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>18:43</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>105</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>17:35:45</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>69</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>17:35:45</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
         <is>
           <t>18:54</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
+      <c r="C180" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D177" t="n">
-        <v>116</v>
-      </c>
-      <c r="E177" t="inlineStr">
+      <c r="D180" t="n">
+        <v>79</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>17:35:45</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>84</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>17:35:45</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>89</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>17:35:45</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>97</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>17:35:45</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>101</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>17:35:45</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>101</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>17:35:45</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>109</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>17:35:45</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>109</v>
+      </c>
+      <c r="E187" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4781,7 +5031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4794,14 +5044,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:58:56</t>
+          <t>Última actualización: 17:35:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5735,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5499,7 +5749,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>46</v>
+        <v>9</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5535,7 +5785,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5549,7 +5799,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -5585,7 +5835,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5599,7 +5849,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -5627,6 +5877,56 @@
         <v>107</v>
       </c>
       <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>17:35:45</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>84</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>17:35:45</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>109</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5643,7 +5943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5656,14 +5956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:58:56</t>
+          <t>Última actualización: 17:35:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -6397,7 +6697,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6411,11 +6711,36 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>106</v>
+        <v>69</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>17:35:45</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>19:14</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>99</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2571
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E187"/>
+  <dimension ref="A1:E193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:35:45</t>
+          <t>Última actualización: 18:06:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 182</t>
+          <t>Total filas: 188</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>18:06:20</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4612,7 +4612,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>107</v>
+        <v>9</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>18:06:20</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,12 +4648,12 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>18:06:20</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>87</v>
+        <v>18</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>18:32</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>57</v>
+        <v>117</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4728,16 +4728,16 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:32</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>18:06:20</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>61</v>
+        <v>28</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:35:45</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>18:43</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>105</v>
+        <v>61</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,12 +4798,12 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:43</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -4812,7 +4812,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>69</v>
+        <v>105</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>18:06:20</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:44</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>79</v>
+        <v>38</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>18:06:20</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>18:59</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>84</v>
+        <v>48</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4878,16 +4878,16 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>18:59</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>18:06:20</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>97</v>
+        <v>58</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>18:06:20</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>101</v>
+        <v>66</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>18:06:20</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>109</v>
+        <v>70</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,23 +4998,173 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
+          <t>18:06:20</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>71</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
           <t>17:35:45</t>
         </is>
       </c>
-      <c r="B187" t="inlineStr">
+      <c r="B188" t="inlineStr">
         <is>
           <t>19:24</t>
         </is>
       </c>
-      <c r="C187" t="inlineStr">
+      <c r="C188" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D187" t="n">
+      <c r="D188" t="n">
         <v>109</v>
       </c>
-      <c r="E187" t="inlineStr">
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>18:06:20</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>78</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>18:06:20</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>79</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>18:06:20</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>103</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>18:06:20</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>104</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>18:06:20</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>109</v>
+      </c>
+      <c r="E193" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5031,7 +5181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5044,14 +5194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:35:45</t>
+          <t>Última actualización: 18:06:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -5860,7 +6010,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>18:06:20</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -5874,7 +6024,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>107</v>
+        <v>9</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -5927,6 +6077,31 @@
         <v>109</v>
       </c>
       <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>18:06:20</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>79</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5943,7 +6118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5956,14 +6131,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:35:45</t>
+          <t>Última actualización: 18:06:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -6722,25 +6897,100 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>18:06:20</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>39</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>17:35:45</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>19:14</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D36" t="n">
         <v>99</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>18:06:20</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>69</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>18:06:20</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>101</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2572
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E193"/>
+  <dimension ref="A1:E200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:06:20</t>
+          <t>Última actualización: 18:48:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 188</t>
+          <t>Total filas: 195</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>18:06:20</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,7 +4873,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>18:06:20</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,12 +4923,12 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>18:06:20</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -4937,7 +4937,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>18:06:20</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>101</v>
+        <v>66</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>18:06:20</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,12 +4998,12 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>18:06:20</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>18:06:20</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>109</v>
+        <v>71</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>18:06:20</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>78</v>
+        <v>36</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>18:06:20</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5103,16 +5103,16 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>18:06:20</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>104</v>
+        <v>61</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,23 +5148,198 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
+          <t>18:48:43</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>62</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
           <t>18:06:20</t>
         </is>
       </c>
-      <c r="B193" t="inlineStr">
+      <c r="B194" t="inlineStr">
         <is>
           <t>19:55</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr">
+      <c r="C194" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D193" t="n">
+      <c r="D194" t="n">
         <v>109</v>
       </c>
-      <c r="E193" t="inlineStr">
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>18:48:43</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>19:56</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>68</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>18:48:43</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>20:11</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>83</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>18:48:43</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>86</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>18:48:43</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>87</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>18:48:43</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>111</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>18:48:43</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>113</v>
+      </c>
+      <c r="E200" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5181,7 +5356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5194,14 +5369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:06:20</t>
+          <t>Última actualización: 18:48:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -6035,7 +6210,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6049,7 +6224,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6060,7 +6235,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6074,7 +6249,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>109</v>
+        <v>36</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6102,6 +6277,56 @@
         <v>79</v>
       </c>
       <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>18:48:43</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>86</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>18:48:43</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>111</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6118,7 +6343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6131,14 +6356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:06:20</t>
+          <t>Última actualización: 18:48:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -6922,7 +7147,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>17:35:45</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6936,7 +7161,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>99</v>
+        <v>26</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6972,23 +7197,73 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>18:48:43</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>58</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>18:06:20</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>19:47</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D39" t="n">
         <v>101</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>18:48:43</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>117</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2573
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E200"/>
+  <dimension ref="A1:E211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:48:44</t>
+          <t>Última actualización: 19:18:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 195</t>
+          <t>Total filas: 206</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,12 +5098,12 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>18:06:20</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -5112,7 +5112,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>61</v>
+        <v>7</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>18:06:20</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>109</v>
+        <v>32</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,12 +5198,12 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>18:06:20</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>19:56</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>68</v>
+        <v>109</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>20:11</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>83</v>
+        <v>38</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5253,16 +5253,16 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:11</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:13</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>87</v>
+        <v>55</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5303,16 +5303,16 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>111</v>
+        <v>86</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,23 +5323,298 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
+          <t>19:18:04</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>56</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>19:18:04</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>57</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
           <t>18:48:43</t>
         </is>
       </c>
-      <c r="B200" t="inlineStr">
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>87</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>19:18:04</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>58</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>18:48:43</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>111</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>19:18:04</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>82</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>18:48:43</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
         <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C200" t="inlineStr">
+      <c r="C206" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D200" t="n">
+      <c r="D206" t="n">
         <v>113</v>
       </c>
-      <c r="E200" t="inlineStr">
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>19:18:04</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>84</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>19:18:04</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>20:53</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>95</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>19:18:04</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>99</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>19:18:04</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>108</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>19:18:04</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>109</v>
+      </c>
+      <c r="E211" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5356,7 +5631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5369,14 +5644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:48:44</t>
+          <t>Última actualización: 19:18:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -6260,7 +6535,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>18:06:20</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6274,7 +6549,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>79</v>
+        <v>7</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -6310,23 +6585,73 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>19:18:04</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>57</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>18:48:43</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>20:39</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D43" t="n">
         <v>111</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>19:18:04</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>82</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6343,7 +6668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6356,14 +6681,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:48:44</t>
+          <t>Última actualización: 19:18:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -7197,37 +7522,37 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>18:06:20</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -7236,7 +7561,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>101</v>
+        <v>58</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -7247,23 +7572,73 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>19:18:04</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>29</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>19:18:04</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>81</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>18:48:43</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>20:45</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="D42" t="n">
         <v>117</v>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2574
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E211"/>
+  <dimension ref="A1:E217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:18:04</t>
+          <t>Última actualización: 19:57:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 206</t>
+          <t>Total filas: 212</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>11:07:13</t>
+          <t>10:21:55</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>10:21:55</t>
+          <t>11:07:13</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:57:10</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>20:11</t>
+          <t>19:57</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>19:57:10</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>20:13</t>
+          <t>20:04</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>55</v>
+        <v>7</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5303,16 +5303,16 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:11</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5328,16 +5328,16 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:13</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,12 +5348,12 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>57</v>
+        <v>86</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>87</v>
+        <v>56</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>19:57:10</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>19:57:10</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:57:10</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>113</v>
+        <v>39</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>19:57:10</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>20:53</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>95</v>
+        <v>43</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>19:57:10</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>108</v>
+        <v>45</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5603,18 +5603,168 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
+          <t>20:53</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>95</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>19:57:10</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>60</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>19:57:10</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>21:01</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>64</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>19:57:10</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>69</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>19:57:10</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
           <t>21:07</t>
         </is>
       </c>
-      <c r="C211" t="inlineStr">
+      <c r="C215" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D211" t="n">
-        <v>109</v>
-      </c>
-      <c r="E211" t="inlineStr">
+      <c r="D215" t="n">
+        <v>70</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>19:57:10</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>97</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>19:57:10</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>100</v>
+      </c>
+      <c r="E217" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5644,7 +5794,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:18:04</t>
+          <t>Última actualización: 19:57:10</t>
         </is>
       </c>
     </row>
@@ -6585,7 +6735,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>19:57:10</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -6599,7 +6749,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>57</v>
+        <v>18</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -6635,7 +6785,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>19:57:10</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -6649,7 +6799,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>82</v>
+        <v>43</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -6668,7 +6818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6681,14 +6831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:18:04</t>
+          <t>Última actualización: 19:57:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -7622,23 +7772,73 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>19:57:10</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>45</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>18:48:43</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>20:45</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D43" t="n">
         <v>117</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>19:57:10</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>95</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2575
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E217"/>
+  <dimension ref="A1:E224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:57:10</t>
+          <t>Última actualización: 20:30:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 212</t>
+          <t>Total filas: 219</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>08:03:30</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:03:30</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>16:28:16</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>16:28:16</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>19:57:10</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>18</v>
+        <v>87</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,7 +5423,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:57:10</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -5433,11 +5433,11 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>87</v>
+        <v>18</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>19:57:10</t>
+          <t>20:30:37</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>20:30:37</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>111</v>
+        <v>9</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>19:57:10</t>
+          <t>20:30:37</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,12 +5598,12 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>20:30:37</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>20:53</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -5612,7 +5612,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>95</v>
+        <v>21</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>19:57:10</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:53</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>60</v>
+        <v>95</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>19:57:10</t>
+          <t>20:30:37</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5678,16 +5678,16 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5703,16 +5703,16 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>21:07</t>
+          <t>21:01</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>19:57:10</t>
+          <t>20:30:37</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>97</v>
+        <v>35</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5753,18 +5753,193 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>69</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>20:30:37</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>37</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>20:30:37</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>64</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>20:30:37</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>66</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>20:30:37</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
           <t>21:37</t>
         </is>
       </c>
-      <c r="C217" t="inlineStr">
+      <c r="C221" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D217" t="n">
-        <v>100</v>
-      </c>
-      <c r="E217" t="inlineStr">
+      <c r="D221" t="n">
+        <v>67</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>20:30:37</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>21:44</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>74</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>20:30:37</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>88</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>20:30:37</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>116</v>
+      </c>
+      <c r="E224" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5794,7 +5969,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:57:10</t>
+          <t>Última actualización: 20:30:37</t>
         </is>
       </c>
     </row>
@@ -6760,7 +6935,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>20:30:37</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -6774,7 +6949,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>111</v>
+        <v>9</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -6818,7 +6993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6831,14 +7006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:57:10</t>
+          <t>Última actualización: 20:30:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -7822,25 +7997,100 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>20:30:37</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>20:48</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>18</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>20:30:37</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>61</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>19:57:10</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>21:32</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D44" t="n">
+      <c r="D46" t="n">
         <v>95</v>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>20:30:37</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>99</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2576
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-19.xlsx
+++ b/data/horarios-141-2026-04-19.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E224"/>
+  <dimension ref="A1:E231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:30:37</t>
+          <t>Última actualización: 21:05:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 219</t>
+          <t>Total filas: 226</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>08:46:39</t>
+          <t>09:04:03</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>09:04:03</t>
+          <t>08:46:39</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:18:04</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>86</v>
+        <v>56</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>19:18:04</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>56</v>
+        <v>86</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>18:48:43</t>
+          <t>19:57:10</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>87</v>
+        <v>18</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,7 +5423,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>19:57:10</t>
+          <t>18:48:43</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -5433,11 +5433,11 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>18</v>
+        <v>87</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>19:57:10</t>
+          <t>21:05:16</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5762,7 +5762,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>20:30:37</t>
+          <t>21:05:16</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5787,7 +5787,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>20:30:37</t>
+          <t>21:05:16</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5812,7 +5812,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>20:30:37</t>
+          <t>21:05:16</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5837,7 +5837,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,7 +5848,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>20:30:37</t>
+          <t>21:05:16</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>67</v>
+        <v>32</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,12 +5873,12 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>20:30:37</t>
+          <t>21:05:16</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>21:44</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -5887,7 +5887,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>74</v>
+        <v>35</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5903,16 +5903,16 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>21:58</t>
+          <t>21:44</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5928,18 +5928,193 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>88</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>21:05:16</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>54</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>21:05:16</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>62</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>21:05:16</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
           <t>22:26</t>
         </is>
       </c>
-      <c r="C224" t="inlineStr">
+      <c r="C227" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D224" t="n">
-        <v>116</v>
-      </c>
-      <c r="E224" t="inlineStr">
+      <c r="D227" t="n">
+        <v>81</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>21:05:16</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>92</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>21:05:16</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>22:41</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>96</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>21:05:16</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>22:53</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>108</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>21:05:16</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>22:56</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>111</v>
+      </c>
+      <c r="E231" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5956,7 +6131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5969,14 +6144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:30:37</t>
+          <t>Última actualización: 21:05:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -6977,6 +7152,31 @@
         <v>43</v>
       </c>
       <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>21:05:16</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>92</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7006,7 +7206,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:30:37</t>
+          <t>Última actualización: 21:05:16</t>
         </is>
       </c>
     </row>
@@ -8047,7 +8247,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19:57:10</t>
+          <t>21:05:16</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8061,7 +8261,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>95</v>
+        <v>27</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8072,7 +8272,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>20:30:37</t>
+          <t>21:05:16</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8086,7 +8286,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>

</xml_diff>